<commit_message>
monitor  I and max E measured
</commit_message>
<xml_diff>
--- a/Kalibrierung_Monitorfaktoren_2025-04-15.xlsx
+++ b/Kalibrierung_Monitorfaktoren_2025-04-15.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Documents\berk\roombrightening\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94C1799F-39E4-4321-9D77-3CCC0E0140CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB000444-8FAF-435E-B643-EAE43061D044}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1845" yWindow="-15870" windowWidth="25440" windowHeight="15270" activeTab="4" xr2:uid="{17DC406C-42B8-4956-9234-CDF5DC26EB7C}"/>
+    <workbookView xWindow="5535" yWindow="-10740" windowWidth="21600" windowHeight="11295" activeTab="4" xr2:uid="{17DC406C-42B8-4956-9234-CDF5DC26EB7C}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -4191,13 +4191,13 @@
       </c>
       <c r="I2" s="1">
         <f xml:space="preserve"> SUM(E3:E5)/3</f>
-        <v>24330240.409480657</v>
+        <v>23290759.748018939</v>
       </c>
       <c r="K2" s="7" t="s">
         <v>27</v>
       </c>
       <c r="L2">
-        <v>170.2</v>
+        <v>174.5</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
@@ -4208,14 +4208,14 @@
         <v>1</v>
       </c>
       <c r="C3" s="1">
-        <v>4.1059999999999998E-8</v>
+        <v>4.2909999999999998E-8</v>
       </c>
       <c r="D3">
         <v>1</v>
       </c>
       <c r="E3" s="1">
         <f>Tabelle15[[#This Row],[E_Measured]]/Tabelle15[[#This Row],[A_Monitor]]</f>
-        <v>24354603.019970775</v>
+        <v>23304591.004427873</v>
       </c>
       <c r="F3">
         <f>Tabelle15[[#This Row],[E_Measured]]/Tabelle15[[#This Row],[E_ideal]]</f>
@@ -4226,13 +4226,13 @@
       </c>
       <c r="I3" s="1">
         <f xml:space="preserve"> SUM(E7:E9)/3</f>
-        <v>27537654.390823841</v>
+        <v>27141303.154015142</v>
       </c>
       <c r="K3" s="7" t="s">
         <v>19</v>
       </c>
       <c r="L3">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
@@ -4243,14 +4243,14 @@
         <v>10</v>
       </c>
       <c r="C4" s="1">
-        <v>4.1189999999999998E-7</v>
+        <v>4.3010000000000002E-7</v>
       </c>
       <c r="D4">
         <v>10.01</v>
       </c>
       <c r="E4" s="1">
         <f>Tabelle15[[#This Row],[E_Measured]]/Tabelle15[[#This Row],[A_Monitor]]</f>
-        <v>24302015.052197136</v>
+        <v>23273657.289002556</v>
       </c>
       <c r="F4">
         <f>Tabelle15[[#This Row],[E_Measured]]/Tabelle15[[#This Row],[E_ideal]]</f>
@@ -4266,14 +4266,14 @@
         <v>31.6</v>
       </c>
       <c r="C5" s="1">
-        <v>1.299E-6</v>
+        <v>1.3570000000000001E-6</v>
       </c>
       <c r="D5">
         <v>31.61</v>
       </c>
       <c r="E5" s="1">
         <f>Tabelle15[[#This Row],[E_Measured]]/Tabelle15[[#This Row],[A_Monitor]]</f>
-        <v>24334103.156274058</v>
+        <v>23294030.950626381</v>
       </c>
       <c r="F5">
         <f>Tabelle15[[#This Row],[E_Measured]]/Tabelle15[[#This Row],[E_ideal]]</f>
@@ -4289,14 +4289,14 @@
         <v>0.1</v>
       </c>
       <c r="C6" s="1">
-        <v>3.476E-9</v>
+        <v>3.565E-9</v>
       </c>
       <c r="D6">
         <v>0.1</v>
       </c>
       <c r="E6" s="1">
         <f>Tabelle15[[#This Row],[E_Measured]]/Tabelle15[[#This Row],[A_Monitor]]</f>
-        <v>28768699.654775605</v>
+        <v>28050490.883590464</v>
       </c>
       <c r="F6">
         <f>Tabelle15[[#This Row],[E_Measured]]/Tabelle15[[#This Row],[E_ideal]]</f>
@@ -4312,14 +4312,14 @@
         <v>1</v>
       </c>
       <c r="C7" s="1">
-        <v>3.6160000000000001E-8</v>
+        <v>3.7009999999999999E-8</v>
       </c>
       <c r="D7">
         <v>1</v>
       </c>
       <c r="E7" s="1">
         <f>Tabelle15[[#This Row],[E_Measured]]/Tabelle15[[#This Row],[A_Monitor]]</f>
-        <v>27654867.256637167</v>
+        <v>27019724.398811132</v>
       </c>
       <c r="F7">
         <f>Tabelle15[[#This Row],[E_Measured]]/Tabelle15[[#This Row],[E_ideal]]</f>
@@ -4334,14 +4334,14 @@
         <v>10</v>
       </c>
       <c r="C8" s="1">
-        <v>3.6469999999999998E-7</v>
+        <v>3.6800000000000001E-7</v>
       </c>
       <c r="D8">
         <v>10.01</v>
       </c>
       <c r="E8" s="1">
         <f>Tabelle15[[#This Row],[E_Measured]]/Tabelle15[[#This Row],[A_Monitor]]</f>
-        <v>27447216.890595011</v>
+        <v>27201086.956521738</v>
       </c>
       <c r="F8">
         <f>Tabelle15[[#This Row],[E_Measured]]/Tabelle15[[#This Row],[E_ideal]]</f>
@@ -4356,14 +4356,14 @@
         <v>31.6</v>
       </c>
       <c r="C9" s="1">
-        <v>1.1489999999999999E-6</v>
+        <v>1.1620000000000001E-6</v>
       </c>
       <c r="D9">
         <v>31.61</v>
       </c>
       <c r="E9" s="1">
         <f>Tabelle15[[#This Row],[E_Measured]]/Tabelle15[[#This Row],[A_Monitor]]</f>
-        <v>27510879.025239341</v>
+        <v>27203098.106712561</v>
       </c>
       <c r="F9">
         <f>Tabelle15[[#This Row],[E_Measured]]/Tabelle15[[#This Row],[E_ideal]]</f>

</xml_diff>

<commit_message>
reading light caused monitor value added to the file
</commit_message>
<xml_diff>
--- a/Kalibrierung_Monitorfaktoren_2025-04-15.xlsx
+++ b/Kalibrierung_Monitorfaktoren_2025-04-15.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Documents\berk\roombrightening\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB000444-8FAF-435E-B643-EAE43061D044}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60F308BC-4046-468E-B11D-CEF7077071FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5535" yWindow="-10740" windowWidth="21600" windowHeight="11295" activeTab="4" xr2:uid="{17DC406C-42B8-4956-9234-CDF5DC26EB7C}"/>
+    <workbookView xWindow="2250" yWindow="-14670" windowWidth="21600" windowHeight="11295" activeTab="4" xr2:uid="{17DC406C-42B8-4956-9234-CDF5DC26EB7C}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="29">
   <si>
     <t>Spot</t>
   </si>
@@ -125,6 +125,9 @@
   </si>
   <si>
     <t>Spot 1 (Only Center)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> because of reading light</t>
   </si>
 </sst>
 </file>
@@ -4125,13 +4128,14 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2FB88217-FE2E-45E2-B182-CE8B986A0E10}">
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="13.7109375" customWidth="1"/>
     <col min="4" max="4" width="16.5703125" customWidth="1"/>
     <col min="5" max="5" width="13.85546875" customWidth="1"/>
     <col min="6" max="6" width="16.140625" customWidth="1"/>
+    <col min="8" max="8" width="14.28515625" customWidth="1"/>
     <col min="9" max="9" width="18.85546875" customWidth="1"/>
     <col min="11" max="11" width="21.42578125" customWidth="1"/>
     <col min="12" max="12" width="14.5703125" customWidth="1"/>
@@ -4325,6 +4329,7 @@
         <f>Tabelle15[[#This Row],[E_Measured]]/Tabelle15[[#This Row],[E_ideal]]</f>
         <v>1</v>
       </c>
+      <c r="H7" s="1"/>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
@@ -4378,6 +4383,14 @@
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>18</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>8.9999999999999999E-10</v>
+      </c>
+      <c r="B15" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>